<commit_message>
Removed the optimal threshold comparison and swapped the Example data for a newer session with the better dynamic range
</commit_message>
<xml_diff>
--- a/Lickometry Data/Example/SensorMap.xlsx
+++ b/Lickometry Data/Example/SensorMap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailuc-my.sharepoint.com/personal/timmens_ucmail_uc_edu/Documents/NickExperimental/HomeCageDrinking/AEW4/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christopher/TimmeLab/CLiQR/Lickometry Data/Example/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{85012687-8B4B-422D-85EB-DFF375BE65AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A8432D7-C305-4184-A594-23409B8F7478}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B6C927E-32D1-E542-942D-837DDA5087B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{FBDA1912-203E-495C-9374-35981934FD62}"/>
+    <workbookView xWindow="-25440" yWindow="-120" windowWidth="25440" windowHeight="15280" xr2:uid="{FBDA1912-203E-495C-9374-35981934FD62}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,72 +36,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
-  <si>
-    <t>AEW4-1</t>
-  </si>
-  <si>
-    <t>AEW4-2</t>
-  </si>
-  <si>
-    <t>AEW4-3</t>
-  </si>
-  <si>
-    <t>AEW4-4</t>
-  </si>
-  <si>
-    <t>AEW4-5</t>
-  </si>
-  <si>
-    <t>AEW4-6</t>
-  </si>
-  <si>
-    <t>AEW4-7</t>
-  </si>
-  <si>
-    <t>AEW4-8</t>
-  </si>
-  <si>
-    <t>AEW4-9</t>
-  </si>
-  <si>
-    <t>AEW4-10</t>
-  </si>
-  <si>
-    <t>AEW4-11</t>
-  </si>
-  <si>
-    <t>AEW4-12</t>
-  </si>
-  <si>
-    <t>AEW4-13</t>
-  </si>
-  <si>
-    <t>AEW4-14</t>
-  </si>
-  <si>
-    <t>AEW4-15</t>
-  </si>
-  <si>
-    <t>AEW4-16</t>
-  </si>
-  <si>
-    <t>AEW4-17</t>
-  </si>
-  <si>
-    <t>AEW4-18</t>
-  </si>
-  <si>
-    <t>AEW4-19</t>
-  </si>
-  <si>
-    <t>AEW4-20</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Drinking Sensor</t>
   </si>
   <si>
     <t>Sipper Label</t>
+  </si>
+  <si>
+    <t>ACG-26-3-1</t>
+  </si>
+  <si>
+    <t>ACG-26-3-2</t>
+  </si>
+  <si>
+    <t>ACG-26-3-3</t>
+  </si>
+  <si>
+    <t>ACG-26-3-4</t>
+  </si>
+  <si>
+    <t>ACG-26-3-5</t>
+  </si>
+  <si>
+    <t>ACG-26-3-6</t>
+  </si>
+  <si>
+    <t>ACG-26-3-7</t>
+  </si>
+  <si>
+    <t>ACG-26-3-8</t>
   </si>
 </sst>
 </file>
@@ -160,10 +124,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -483,179 +443,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41E0F3C-5C31-4BB7-92CF-EDA1048F76AB}">
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
-    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="2" max="2" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B9">
         <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>